<commit_message>
Add updated docs for iteration 3; Update README.md with deployment details.
</commit_message>
<xml_diff>
--- a/doc/CS673_SPPP_RiskManagement.xlsx
+++ b/doc/CS673_SPPP_RiskManagement.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="n3I/BP8fEBL3b256mabHaNL+tJbfgF2697wUf85UM6c="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="rZTng+sYipBIzWrI2IIBekmDXRiu7q6bhdnIjB/TYM4="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="130">
   <si>
     <t>This sheet provides some common risks in student projects. You should check if it applies to your group project. 
 You should also feel free to add other risks. Exemplary analysis is also added.</t>
@@ -110,6 +110,24 @@
     <t>Lack of motivation or responsibility</t>
   </si>
   <si>
+    <t>Missed deadlines</t>
+  </si>
+  <si>
+    <t>Documents and code merges done after deadlines</t>
+  </si>
+  <si>
+    <t>Team leader and all members</t>
+  </si>
+  <si>
+    <t>Message members with reminders about deadlines. Tell members about deadlines during meetings. Make members verbally confirm deadlines.</t>
+  </si>
+  <si>
+    <t>Last deadline had significantly less last-minute code then previous deadlines. However, some code was still submitted after deadline and thus was not merged</t>
+  </si>
+  <si>
+    <t>closed</t>
+  </si>
+  <si>
     <t>Communication</t>
   </si>
   <si>
@@ -149,6 +167,9 @@
     <t>Bring up at next meeting</t>
   </si>
   <si>
+    <t>Despite reminders, continues to be a problem</t>
+  </si>
+  <si>
     <t xml:space="preserve">Requirements </t>
   </si>
   <si>
@@ -372,6 +393,21 @@
   </si>
   <si>
     <t>Educate the team on code review strategy. Enforce atleast 2 reviewers per PR</t>
+  </si>
+  <si>
+    <t>Lack of code reviews</t>
+  </si>
+  <si>
+    <t>PRs go several days without being reviewed, causing code not to be merged until weeks after it was written</t>
+  </si>
+  <si>
+    <t>All members</t>
+  </si>
+  <si>
+    <t>Assign specific members to specific pull requests. Reduce required reviews to 1.</t>
+  </si>
+  <si>
+    <t>Reducing reviews to 1 increase the speed of PRs being merged, but the amount of reviews has failed to increase</t>
   </si>
   <si>
     <t>The team member who is adding the new feature should be the one who determines what is correct for the new functionality that was added.</t>
@@ -388,7 +424,7 @@
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="165" formatCode="m/d"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -402,6 +438,11 @@
     <font>
       <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <color rgb="FF000000"/>
@@ -434,7 +475,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="24">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -459,13 +500,15 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
@@ -478,7 +521,8 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -489,6 +533,18 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -700,6 +756,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
@@ -823,30 +880,30 @@
       <c r="AA3" s="7"/>
     </row>
     <row r="4">
-      <c r="A4" s="3"/>
+      <c r="A4" s="8"/>
       <c r="B4" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="9">
         <v>2.0</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="9">
         <v>3.0</v>
       </c>
-      <c r="F4" s="8">
+      <c r="F4" s="9">
         <v>3.0</v>
       </c>
-      <c r="G4" s="8">
-        <f t="shared" ref="G4:G23" si="1">D4*E4*F4</f>
+      <c r="G4" s="9">
+        <f t="shared" ref="G4:G24" si="1">D4*E4*F4</f>
         <v>18</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="9">
+      <c r="I4" s="10">
         <v>45922.0</v>
       </c>
       <c r="J4" s="3" t="s">
@@ -880,14 +937,14 @@
         <v>27</v>
       </c>
       <c r="C5" s="3"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8">
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I5" s="9"/>
+      <c r="I5" s="10"/>
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
       <c r="L5" s="3"/>
@@ -908,25 +965,41 @@
       <c r="AA5" s="7"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="3"/>
+      <c r="B6" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8">
+      <c r="D6" s="13">
+        <v>5.0</v>
+      </c>
+      <c r="E6" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="F6" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="G6" s="9">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H6" s="3"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
+        <v>30</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" s="14">
+        <v>45988.0</v>
+      </c>
+      <c r="J6" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="K6" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L6" s="12" t="s">
+        <v>33</v>
+      </c>
       <c r="M6" s="7"/>
       <c r="N6" s="7"/>
       <c r="O6" s="7"/>
@@ -944,39 +1017,25 @@
       <c r="AA6" s="7"/>
     </row>
     <row r="7">
-      <c r="A7" s="2"/>
+      <c r="A7" s="3" t="s">
+        <v>34</v>
+      </c>
       <c r="B7" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D7" s="8">
-        <v>2.0</v>
-      </c>
-      <c r="E7" s="8">
-        <v>4.0</v>
-      </c>
-      <c r="F7" s="8">
-        <v>2.0</v>
-      </c>
-      <c r="G7" s="8">
+        <v>35</v>
+      </c>
+      <c r="C7" s="3"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9">
         <f t="shared" si="1"/>
-        <v>16</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="I7" s="9">
-        <v>45995.0</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>33</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H7" s="3"/>
+      <c r="I7" s="10"/>
+      <c r="J7" s="3"/>
       <c r="K7" s="3"/>
-      <c r="L7" s="3" t="s">
-        <v>26</v>
-      </c>
+      <c r="L7" s="3"/>
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
@@ -994,34 +1053,34 @@
       <c r="AA7" s="7"/>
     </row>
     <row r="8">
-      <c r="A8" s="3"/>
+      <c r="A8" s="2"/>
       <c r="B8" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D8" s="8">
+        <v>37</v>
+      </c>
+      <c r="D8" s="9">
         <v>2.0</v>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="9">
         <v>4.0</v>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="9">
         <v>2.0</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="9">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I8" s="9">
+        <v>38</v>
+      </c>
+      <c r="I8" s="10">
         <v>45995.0</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="K8" s="3"/>
       <c r="L8" s="3" t="s">
@@ -1045,22 +1104,38 @@
     </row>
     <row r="9">
       <c r="A9" s="3"/>
-      <c r="B9" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8">
+      <c r="B9" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D9" s="9">
+        <v>2.0</v>
+      </c>
+      <c r="E9" s="9">
+        <v>4.0</v>
+      </c>
+      <c r="F9" s="9">
+        <v>2.0</v>
+      </c>
+      <c r="G9" s="9">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H9" s="3"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="3"/>
+        <v>16</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="I9" s="10">
+        <v>45995.0</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>42</v>
+      </c>
       <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
+      <c r="L9" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="M9" s="7"/>
       <c r="N9" s="7"/>
       <c r="O9" s="7"/>
@@ -1079,38 +1154,22 @@
     </row>
     <row r="10">
       <c r="A10" s="3"/>
-      <c r="B10" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D10" s="8">
-        <v>4.0</v>
-      </c>
-      <c r="E10" s="8">
-        <v>3.0</v>
-      </c>
-      <c r="F10" s="8">
-        <v>3.0</v>
-      </c>
-      <c r="G10" s="8">
+      <c r="B10" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9">
         <f t="shared" si="1"/>
-        <v>36</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I10" s="9">
-        <v>45932.0</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H10" s="3"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="3"/>
       <c r="K10" s="3"/>
-      <c r="L10" s="3" t="s">
-        <v>26</v>
-      </c>
+      <c r="L10" s="3"/>
       <c r="M10" s="7"/>
       <c r="N10" s="7"/>
       <c r="O10" s="7"/>
@@ -1128,38 +1187,38 @@
       <c r="AA10" s="7"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>42</v>
+      <c r="A11" s="3"/>
+      <c r="B11" s="15" t="s">
+        <v>44</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="D11" s="8">
-        <v>2.0</v>
-      </c>
-      <c r="E11" s="8">
+        <v>45</v>
+      </c>
+      <c r="D11" s="9">
+        <v>4.0</v>
+      </c>
+      <c r="E11" s="9">
         <v>3.0</v>
       </c>
-      <c r="F11" s="8">
-        <v>4.0</v>
-      </c>
-      <c r="G11" s="8">
+      <c r="F11" s="9">
+        <v>3.0</v>
+      </c>
+      <c r="G11" s="9">
         <f t="shared" si="1"/>
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I11" s="9">
-        <v>45995.0</v>
+      <c r="I11" s="10">
+        <v>45932.0</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="K11" s="3"/>
+        <v>46</v>
+      </c>
+      <c r="K11" s="12" t="s">
+        <v>47</v>
+      </c>
       <c r="L11" s="3" t="s">
         <v>26</v>
       </c>
@@ -1180,23 +1239,41 @@
       <c r="AA11" s="7"/>
     </row>
     <row r="12">
-      <c r="A12" s="3"/>
+      <c r="A12" s="3" t="s">
+        <v>48</v>
+      </c>
       <c r="B12" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C12" s="3"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8">
+        <v>49</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" s="9">
+        <v>2.0</v>
+      </c>
+      <c r="E12" s="9">
+        <v>3.0</v>
+      </c>
+      <c r="F12" s="9">
+        <v>4.0</v>
+      </c>
+      <c r="G12" s="9">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H12" s="3"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="3"/>
+        <v>24</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="I12" s="10">
+        <v>45995.0</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>51</v>
+      </c>
       <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
+      <c r="L12" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="M12" s="7"/>
       <c r="N12" s="7"/>
       <c r="O12" s="7"/>
@@ -1216,18 +1293,18 @@
     <row r="13">
       <c r="A13" s="3"/>
       <c r="B13" s="2" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="C13" s="3"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8">
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="H13" s="3"/>
-      <c r="I13" s="9"/>
+      <c r="I13" s="10"/>
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
       <c r="L13" s="3"/>
@@ -1248,41 +1325,23 @@
       <c r="AA13" s="7"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="s">
-        <v>47</v>
-      </c>
+      <c r="A14" s="3"/>
       <c r="B14" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="D14" s="8">
-        <v>3.0</v>
-      </c>
-      <c r="E14" s="8">
-        <v>4.0</v>
-      </c>
-      <c r="F14" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="G14" s="8">
+        <v>53</v>
+      </c>
+      <c r="C14" s="3"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9">
         <f t="shared" si="1"/>
-        <v>12</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="I14" s="9"/>
-      <c r="J14" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="K14" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="L14" s="3" t="s">
-        <v>26</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H14" s="3"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
       <c r="M14" s="7"/>
       <c r="N14" s="7"/>
       <c r="O14" s="7"/>
@@ -1300,35 +1359,37 @@
       <c r="AA14" s="7"/>
     </row>
     <row r="15">
-      <c r="A15" s="3"/>
+      <c r="A15" s="3" t="s">
+        <v>54</v>
+      </c>
       <c r="B15" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="D15" s="8">
-        <v>2.0</v>
-      </c>
-      <c r="E15" s="8">
+        <v>56</v>
+      </c>
+      <c r="D15" s="9">
+        <v>3.0</v>
+      </c>
+      <c r="E15" s="9">
         <v>4.0</v>
       </c>
-      <c r="F15" s="8">
-        <v>3.0</v>
-      </c>
-      <c r="G15" s="8">
+      <c r="F15" s="9">
+        <v>1.0</v>
+      </c>
+      <c r="G15" s="9">
         <f t="shared" si="1"/>
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="I15" s="9"/>
+        <v>57</v>
+      </c>
+      <c r="I15" s="10"/>
       <c r="J15" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="L15" s="3" t="s">
         <v>26</v>
@@ -1351,36 +1412,34 @@
     </row>
     <row r="16">
       <c r="A16" s="3"/>
-      <c r="B16" s="10" t="s">
-        <v>58</v>
+      <c r="B16" s="2" t="s">
+        <v>60</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D16" s="8">
+        <v>61</v>
+      </c>
+      <c r="D16" s="9">
+        <v>2.0</v>
+      </c>
+      <c r="E16" s="9">
         <v>4.0</v>
       </c>
-      <c r="E16" s="8">
-        <v>2.0</v>
-      </c>
-      <c r="F16" s="8">
-        <v>1.0</v>
-      </c>
-      <c r="G16" s="8">
+      <c r="F16" s="9">
+        <v>3.0</v>
+      </c>
+      <c r="G16" s="9">
         <f t="shared" si="1"/>
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="I16" s="9">
-        <v>45918.0</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="I16" s="10"/>
       <c r="J16" s="3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="L16" s="3" t="s">
         <v>26</v>
@@ -1402,40 +1461,40 @@
       <c r="AA16" s="7"/>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="D17" s="13">
+      <c r="A17" s="3"/>
+      <c r="B17" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D17" s="9">
+        <v>4.0</v>
+      </c>
+      <c r="E17" s="9">
         <v>2.0</v>
       </c>
-      <c r="E17" s="13">
-        <v>4.0</v>
-      </c>
-      <c r="F17" s="13">
-        <v>4.0</v>
-      </c>
-      <c r="G17" s="8">
+      <c r="F17" s="9">
+        <v>1.0</v>
+      </c>
+      <c r="G17" s="9">
         <f t="shared" si="1"/>
-        <v>32</v>
-      </c>
-      <c r="H17" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="I17" s="14">
-        <v>45946.0</v>
-      </c>
-      <c r="J17" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="K17" s="3"/>
+        <v>8</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="I17" s="10">
+        <v>45918.0</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>68</v>
+      </c>
       <c r="L17" s="12" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="M17" s="7"/>
       <c r="N17" s="7"/>
@@ -1454,23 +1513,41 @@
       <c r="AA17" s="7"/>
     </row>
     <row r="18">
-      <c r="A18" s="3"/>
+      <c r="A18" s="3" t="s">
+        <v>69</v>
+      </c>
       <c r="B18" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C18" s="3"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8">
+        <v>70</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D18" s="9">
+        <v>2.0</v>
+      </c>
+      <c r="E18" s="9">
+        <v>4.0</v>
+      </c>
+      <c r="F18" s="9">
+        <v>4.0</v>
+      </c>
+      <c r="G18" s="9">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H18" s="3"/>
-      <c r="I18" s="9"/>
-      <c r="J18" s="3"/>
+        <v>32</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="I18" s="10">
+        <v>45946.0</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
+      <c r="L18" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="M18" s="7"/>
       <c r="N18" s="7"/>
       <c r="O18" s="7"/>
@@ -1490,18 +1567,18 @@
     <row r="19">
       <c r="A19" s="3"/>
       <c r="B19" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C19" s="3"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8">
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="H19" s="3"/>
-      <c r="I19" s="9"/>
+      <c r="I19" s="10"/>
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
       <c r="L19" s="3"/>
@@ -1524,18 +1601,18 @@
     <row r="20">
       <c r="A20" s="3"/>
       <c r="B20" s="2" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="C20" s="3"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8">
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="H20" s="3"/>
-      <c r="I20" s="9"/>
+      <c r="I20" s="10"/>
       <c r="J20" s="3"/>
       <c r="K20" s="3"/>
       <c r="L20" s="3"/>
@@ -1558,18 +1635,18 @@
     <row r="21">
       <c r="A21" s="3"/>
       <c r="B21" s="2" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="C21" s="3"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8">
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="H21" s="3"/>
-      <c r="I21" s="9"/>
+      <c r="I21" s="10"/>
       <c r="J21" s="3"/>
       <c r="K21" s="3"/>
       <c r="L21" s="3"/>
@@ -1590,43 +1667,23 @@
       <c r="AA21" s="7"/>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="s">
-        <v>71</v>
-      </c>
+      <c r="A22" s="3"/>
       <c r="B22" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="D22" s="8">
-        <v>2.0</v>
-      </c>
-      <c r="E22" s="8">
-        <v>4.0</v>
-      </c>
-      <c r="F22" s="8">
-        <v>3.0</v>
-      </c>
-      <c r="G22" s="8">
+        <v>77</v>
+      </c>
+      <c r="C22" s="3"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9">
         <f t="shared" si="1"/>
-        <v>24</v>
-      </c>
-      <c r="H22" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="I22" s="9">
-        <v>45995.0</v>
-      </c>
-      <c r="J22" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="K22" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="L22" s="3" t="s">
-        <v>26</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H22" s="3"/>
+      <c r="I22" s="10"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
       <c r="M22" s="7"/>
       <c r="N22" s="7"/>
       <c r="O22" s="7"/>
@@ -1644,37 +1701,39 @@
       <c r="AA22" s="7"/>
     </row>
     <row r="23">
-      <c r="A23" s="3"/>
+      <c r="A23" s="3" t="s">
+        <v>78</v>
+      </c>
       <c r="B23" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D23" s="8">
+        <v>80</v>
+      </c>
+      <c r="D23" s="9">
         <v>2.0</v>
       </c>
-      <c r="E23" s="8">
+      <c r="E23" s="9">
         <v>4.0</v>
       </c>
-      <c r="F23" s="8">
-        <v>4.0</v>
-      </c>
-      <c r="G23" s="8">
+      <c r="F23" s="9">
+        <v>3.0</v>
+      </c>
+      <c r="G23" s="9">
         <f t="shared" si="1"/>
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="I23" s="9">
-        <v>45932.0</v>
+        <v>81</v>
+      </c>
+      <c r="I23" s="10">
+        <v>45995.0</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="L23" s="3" t="s">
         <v>26</v>
@@ -1698,29 +1757,35 @@
     <row r="24">
       <c r="A24" s="3"/>
       <c r="B24" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="D24" s="8">
+        <v>85</v>
+      </c>
+      <c r="D24" s="9">
         <v>2.0</v>
       </c>
-      <c r="E24" s="8">
+      <c r="E24" s="9">
         <v>4.0</v>
       </c>
-      <c r="F24" s="8">
+      <c r="F24" s="9">
         <v>4.0</v>
       </c>
-      <c r="G24" s="8"/>
+      <c r="G24" s="9">
+        <f t="shared" si="1"/>
+        <v>32</v>
+      </c>
       <c r="H24" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="I24" s="9">
-        <v>45995.0</v>
+        <v>86</v>
+      </c>
+      <c r="I24" s="10">
+        <v>45932.0</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
+      </c>
+      <c r="K24" s="3" t="s">
+        <v>88</v>
       </c>
       <c r="L24" s="3" t="s">
         <v>26</v>
@@ -1744,32 +1809,29 @@
     <row r="25">
       <c r="A25" s="3"/>
       <c r="B25" s="2" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C25" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="D25" s="9">
+        <v>2.0</v>
+      </c>
+      <c r="E25" s="9">
+        <v>4.0</v>
+      </c>
+      <c r="F25" s="9">
+        <v>4.0</v>
+      </c>
+      <c r="G25" s="9"/>
+      <c r="H25" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="D25" s="8">
-        <v>2.0</v>
-      </c>
-      <c r="E25" s="8">
-        <v>3.0</v>
-      </c>
-      <c r="F25" s="8">
-        <v>3.0</v>
-      </c>
-      <c r="G25" s="8">
-        <f t="shared" ref="G25:G31" si="2">D25*E25*F25</f>
-        <v>18</v>
-      </c>
-      <c r="H25" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="I25" s="9">
+      <c r="I25" s="10">
         <v>45995.0</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="L25" s="3" t="s">
         <v>26</v>
@@ -1791,39 +1853,34 @@
       <c r="AA25" s="7"/>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="s">
-        <v>89</v>
-      </c>
+      <c r="A26" s="3"/>
       <c r="B26" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="D26" s="8">
+        <v>93</v>
+      </c>
+      <c r="D26" s="9">
+        <v>2.0</v>
+      </c>
+      <c r="E26" s="9">
         <v>3.0</v>
       </c>
-      <c r="E26" s="8">
-        <v>4.0</v>
-      </c>
-      <c r="F26" s="8">
-        <v>2.0</v>
-      </c>
-      <c r="G26" s="8">
-        <f t="shared" si="2"/>
-        <v>24</v>
+      <c r="F26" s="9">
+        <v>3.0</v>
+      </c>
+      <c r="G26" s="9">
+        <f t="shared" ref="G26:G33" si="2">D26*E26*F26</f>
+        <v>18</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="I26" s="9">
+        <v>94</v>
+      </c>
+      <c r="I26" s="10">
         <v>45995.0</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="K26" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="L26" s="3" t="s">
         <v>26</v>
@@ -1846,24 +1903,42 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="B27" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="C27" s="3"/>
-      <c r="D27" s="8"/>
-      <c r="E27" s="8"/>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8">
+      <c r="B27" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D27" s="9">
+        <v>3.0</v>
+      </c>
+      <c r="E27" s="9">
+        <v>4.0</v>
+      </c>
+      <c r="F27" s="9">
+        <v>2.0</v>
+      </c>
+      <c r="G27" s="9">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H27" s="3"/>
-      <c r="I27" s="9"/>
-      <c r="J27" s="3"/>
-      <c r="K27" s="3"/>
-      <c r="L27" s="3"/>
+        <v>24</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="I27" s="10">
+        <v>45995.0</v>
+      </c>
+      <c r="J27" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="K27" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="L27" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="M27" s="7"/>
       <c r="N27" s="7"/>
       <c r="O27" s="7"/>
@@ -1881,43 +1956,25 @@
       <c r="AA27" s="7"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="D28" s="8">
-        <v>2.0</v>
-      </c>
-      <c r="E28" s="8">
-        <v>4.0</v>
-      </c>
-      <c r="F28" s="8">
-        <v>4.0</v>
-      </c>
-      <c r="G28" s="8">
+      <c r="A28" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B28" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="C28" s="3"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
+      <c r="G28" s="9">
         <f t="shared" si="2"/>
-        <v>32</v>
-      </c>
-      <c r="H28" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="I28" s="9">
-        <v>45930.0</v>
-      </c>
-      <c r="J28" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="K28" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="L28" s="3" t="s">
-        <v>26</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H28" s="3"/>
+      <c r="I28" s="10"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
       <c r="M28" s="7"/>
       <c r="N28" s="7"/>
       <c r="O28" s="7"/>
@@ -1935,41 +1992,41 @@
       <c r="AA28" s="7"/>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="B29" s="10" t="s">
+      <c r="A29" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C29" s="7" t="s">
+      <c r="B29" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="D29" s="16">
-        <v>3.0</v>
-      </c>
-      <c r="E29" s="16">
-        <v>5.0</v>
-      </c>
-      <c r="F29" s="16">
-        <v>3.0</v>
-      </c>
-      <c r="G29" s="8">
+      <c r="C29" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="D29" s="9">
+        <v>2.0</v>
+      </c>
+      <c r="E29" s="9">
+        <v>4.0</v>
+      </c>
+      <c r="F29" s="9">
+        <v>4.0</v>
+      </c>
+      <c r="G29" s="9">
         <f t="shared" si="2"/>
-        <v>45</v>
-      </c>
-      <c r="H29" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="I29" s="17">
-        <v>45976.0</v>
-      </c>
-      <c r="J29" s="18" t="s">
-        <v>106</v>
-      </c>
-      <c r="K29" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="H29" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="L29" s="7" t="s">
+      <c r="I29" s="10">
+        <v>45930.0</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="K29" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="L29" s="3" t="s">
         <v>26</v>
       </c>
       <c r="M29" s="7"/>
@@ -1990,38 +2047,38 @@
     </row>
     <row r="30">
       <c r="A30" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="B30" s="10" t="s">
-        <v>109</v>
+        <v>110</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>111</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D30" s="16">
-        <v>2.0</v>
-      </c>
-      <c r="E30" s="16">
+        <v>112</v>
+      </c>
+      <c r="D30" s="17">
+        <v>3.0</v>
+      </c>
+      <c r="E30" s="17">
         <v>5.0</v>
       </c>
-      <c r="F30" s="16">
-        <v>4.0</v>
-      </c>
-      <c r="G30" s="8">
+      <c r="F30" s="17">
+        <v>3.0</v>
+      </c>
+      <c r="G30" s="9">
         <f t="shared" si="2"/>
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="I30" s="17">
-        <v>45960.0</v>
-      </c>
-      <c r="J30" s="7" t="s">
-        <v>111</v>
+        <v>107</v>
+      </c>
+      <c r="I30" s="18">
+        <v>45976.0</v>
+      </c>
+      <c r="J30" s="19" t="s">
+        <v>113</v>
       </c>
       <c r="K30" s="7" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="L30" s="7" t="s">
         <v>26</v>
@@ -2044,38 +2101,38 @@
     </row>
     <row r="31">
       <c r="A31" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="B31" s="10" t="s">
-        <v>113</v>
+        <v>115</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>116</v>
       </c>
       <c r="C31" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="D31" s="17">
+        <v>2.0</v>
+      </c>
+      <c r="E31" s="17">
+        <v>5.0</v>
+      </c>
+      <c r="F31" s="17">
+        <v>4.0</v>
+      </c>
+      <c r="G31" s="9">
+        <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
+      <c r="H31" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="I31" s="18">
+        <v>45960.0</v>
+      </c>
+      <c r="J31" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="K31" s="7" t="s">
         <v>114</v>
-      </c>
-      <c r="D31" s="16">
-        <v>2.0</v>
-      </c>
-      <c r="E31" s="16">
-        <v>4.0</v>
-      </c>
-      <c r="F31" s="16">
-        <v>2.0</v>
-      </c>
-      <c r="G31" s="8">
-        <f t="shared" si="2"/>
-        <v>16</v>
-      </c>
-      <c r="H31" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="I31" s="17">
-        <v>45945.0</v>
-      </c>
-      <c r="J31" s="18" t="s">
-        <v>115</v>
-      </c>
-      <c r="K31" s="7" t="s">
-        <v>107</v>
       </c>
       <c r="L31" s="7" t="s">
         <v>26</v>
@@ -2096,18 +2153,44 @@
       <c r="Z31" s="7"/>
       <c r="AA31" s="7"/>
     </row>
-    <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="7"/>
-      <c r="C32" s="7"/>
-      <c r="D32" s="16"/>
-      <c r="E32" s="16"/>
-      <c r="F32" s="16"/>
-      <c r="G32" s="16"/>
-      <c r="H32" s="7"/>
-      <c r="I32" s="17"/>
-      <c r="J32" s="18"/>
-      <c r="K32" s="7"/>
-      <c r="L32" s="7"/>
+    <row r="32">
+      <c r="A32" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="B32" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="D32" s="17">
+        <v>2.0</v>
+      </c>
+      <c r="E32" s="17">
+        <v>4.0</v>
+      </c>
+      <c r="F32" s="17">
+        <v>2.0</v>
+      </c>
+      <c r="G32" s="9">
+        <f t="shared" si="2"/>
+        <v>16</v>
+      </c>
+      <c r="H32" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="I32" s="18">
+        <v>45945.0</v>
+      </c>
+      <c r="J32" s="19" t="s">
+        <v>122</v>
+      </c>
+      <c r="K32" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="L32" s="7" t="s">
+        <v>26</v>
+      </c>
       <c r="M32" s="7"/>
       <c r="N32" s="7"/>
       <c r="O32" s="7"/>
@@ -2126,16 +2209,40 @@
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="7"/>
-      <c r="C33" s="7"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="16"/>
-      <c r="G33" s="16"/>
-      <c r="H33" s="7"/>
-      <c r="I33" s="17"/>
-      <c r="J33" s="18"/>
-      <c r="K33" s="7"/>
-      <c r="L33" s="7"/>
+      <c r="B33" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="C33" s="20" t="s">
+        <v>124</v>
+      </c>
+      <c r="D33" s="21">
+        <v>3.0</v>
+      </c>
+      <c r="E33" s="21">
+        <v>3.0</v>
+      </c>
+      <c r="F33" s="21">
+        <v>3.0</v>
+      </c>
+      <c r="G33" s="9">
+        <f t="shared" si="2"/>
+        <v>27</v>
+      </c>
+      <c r="H33" s="20" t="s">
+        <v>125</v>
+      </c>
+      <c r="I33" s="22">
+        <v>45995.0</v>
+      </c>
+      <c r="J33" s="23" t="s">
+        <v>126</v>
+      </c>
+      <c r="K33" s="20" t="s">
+        <v>127</v>
+      </c>
+      <c r="L33" s="20" t="s">
+        <v>26</v>
+      </c>
       <c r="M33" s="7"/>
       <c r="N33" s="7"/>
       <c r="O33" s="7"/>
@@ -2155,13 +2262,13 @@
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="7"/>
       <c r="C34" s="7"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="16"/>
-      <c r="F34" s="16"/>
-      <c r="G34" s="16"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="17"/>
+      <c r="G34" s="17"/>
       <c r="H34" s="7"/>
-      <c r="I34" s="17"/>
-      <c r="J34" s="18"/>
+      <c r="I34" s="18"/>
+      <c r="J34" s="19"/>
       <c r="K34" s="7"/>
       <c r="L34" s="7"/>
       <c r="M34" s="7"/>
@@ -2183,13 +2290,13 @@
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="7"/>
       <c r="C35" s="7"/>
-      <c r="D35" s="16"/>
-      <c r="E35" s="16"/>
-      <c r="F35" s="16"/>
-      <c r="G35" s="16"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="17"/>
+      <c r="F35" s="17"/>
+      <c r="G35" s="17"/>
       <c r="H35" s="7"/>
-      <c r="I35" s="17"/>
-      <c r="J35" s="18"/>
+      <c r="I35" s="18"/>
+      <c r="J35" s="19"/>
       <c r="K35" s="7"/>
       <c r="L35" s="7"/>
       <c r="M35" s="7"/>
@@ -2210,15 +2317,14 @@
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="7"/>
-      <c r="B36" s="7"/>
       <c r="C36" s="7"/>
-      <c r="D36" s="7"/>
-      <c r="E36" s="7"/>
-      <c r="F36" s="7"/>
-      <c r="G36" s="7"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="17"/>
+      <c r="F36" s="17"/>
+      <c r="G36" s="17"/>
       <c r="H36" s="7"/>
-      <c r="I36" s="7"/>
-      <c r="J36" s="7"/>
+      <c r="I36" s="18"/>
+      <c r="J36" s="19"/>
       <c r="K36" s="7"/>
       <c r="L36" s="7"/>
       <c r="M36" s="7"/>
@@ -2238,16 +2344,16 @@
       <c r="AA36" s="7"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="3"/>
-      <c r="B37" s="3"/>
-      <c r="C37" s="3"/>
-      <c r="D37" s="16"/>
-      <c r="E37" s="16"/>
-      <c r="F37" s="16"/>
+      <c r="A37" s="7"/>
+      <c r="B37" s="7"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="7"/>
       <c r="G37" s="7"/>
       <c r="H37" s="7"/>
       <c r="I37" s="7"/>
-      <c r="J37" s="3"/>
+      <c r="J37" s="7"/>
       <c r="K37" s="7"/>
       <c r="L37" s="7"/>
       <c r="M37" s="7"/>
@@ -2270,9 +2376,9 @@
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
-      <c r="D38" s="16"/>
-      <c r="E38" s="16"/>
-      <c r="F38" s="16"/>
+      <c r="D38" s="17"/>
+      <c r="E38" s="17"/>
+      <c r="F38" s="17"/>
       <c r="G38" s="7"/>
       <c r="H38" s="7"/>
       <c r="I38" s="7"/>
@@ -2299,9 +2405,9 @@
       <c r="A39" s="3"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
-      <c r="D39" s="16"/>
-      <c r="E39" s="16"/>
-      <c r="F39" s="16"/>
+      <c r="D39" s="17"/>
+      <c r="E39" s="17"/>
+      <c r="F39" s="17"/>
       <c r="G39" s="7"/>
       <c r="H39" s="7"/>
       <c r="I39" s="7"/>
@@ -2328,9 +2434,9 @@
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
-      <c r="D40" s="16"/>
-      <c r="E40" s="16"/>
-      <c r="F40" s="16"/>
+      <c r="D40" s="17"/>
+      <c r="E40" s="17"/>
+      <c r="F40" s="17"/>
       <c r="G40" s="7"/>
       <c r="H40" s="7"/>
       <c r="I40" s="7"/>
@@ -2355,15 +2461,15 @@
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="3"/>
-      <c r="D41" s="16"/>
-      <c r="E41" s="16"/>
-      <c r="F41" s="16"/>
+      <c r="B41" s="3"/>
+      <c r="C41" s="3"/>
+      <c r="D41" s="17"/>
+      <c r="E41" s="17"/>
+      <c r="F41" s="17"/>
       <c r="G41" s="7"/>
       <c r="H41" s="7"/>
       <c r="I41" s="7"/>
-      <c r="J41" s="3" t="s">
-        <v>116</v>
-      </c>
+      <c r="J41" s="3"/>
       <c r="K41" s="7"/>
       <c r="L41" s="7"/>
       <c r="M41" s="7"/>
@@ -2384,16 +2490,14 @@
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="3"/>
-      <c r="B42" s="3"/>
-      <c r="C42" s="3"/>
-      <c r="D42" s="16"/>
-      <c r="E42" s="16"/>
-      <c r="F42" s="16"/>
+      <c r="D42" s="17"/>
+      <c r="E42" s="17"/>
+      <c r="F42" s="17"/>
       <c r="G42" s="7"/>
       <c r="H42" s="7"/>
       <c r="I42" s="7"/>
       <c r="J42" s="3" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="K42" s="7"/>
       <c r="L42" s="7"/>
@@ -2417,13 +2521,15 @@
       <c r="A43" s="3"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
-      <c r="D43" s="16"/>
-      <c r="E43" s="7"/>
-      <c r="F43" s="7"/>
+      <c r="D43" s="17"/>
+      <c r="E43" s="17"/>
+      <c r="F43" s="17"/>
       <c r="G43" s="7"/>
       <c r="H43" s="7"/>
       <c r="I43" s="7"/>
-      <c r="J43" s="3"/>
+      <c r="J43" s="3" t="s">
+        <v>129</v>
+      </c>
       <c r="K43" s="7"/>
       <c r="L43" s="7"/>
       <c r="M43" s="7"/>
@@ -2443,16 +2549,16 @@
       <c r="AA43" s="7"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="A44" s="7"/>
-      <c r="B44" s="7"/>
-      <c r="C44" s="7"/>
-      <c r="D44" s="7"/>
+      <c r="A44" s="3"/>
+      <c r="B44" s="3"/>
+      <c r="C44" s="3"/>
+      <c r="D44" s="17"/>
       <c r="E44" s="7"/>
       <c r="F44" s="7"/>
       <c r="G44" s="7"/>
       <c r="H44" s="7"/>
       <c r="I44" s="7"/>
-      <c r="J44" s="7"/>
+      <c r="J44" s="3"/>
       <c r="K44" s="7"/>
       <c r="L44" s="7"/>
       <c r="M44" s="7"/>
@@ -2471,47 +2577,47 @@
       <c r="Z44" s="7"/>
       <c r="AA44" s="7"/>
     </row>
-    <row r="45" ht="15.75" customHeight="1"/>
-    <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="7"/>
-      <c r="B46" s="7"/>
-      <c r="C46" s="3"/>
-      <c r="D46" s="16"/>
-      <c r="E46" s="16"/>
-      <c r="F46" s="7"/>
-      <c r="G46" s="16"/>
-      <c r="H46" s="7"/>
-      <c r="I46" s="7"/>
-      <c r="J46" s="18"/>
-      <c r="K46" s="7"/>
-      <c r="L46" s="7"/>
-      <c r="M46" s="7"/>
-      <c r="N46" s="7"/>
-      <c r="O46" s="7"/>
-      <c r="P46" s="7"/>
-      <c r="Q46" s="7"/>
-      <c r="R46" s="7"/>
-      <c r="S46" s="7"/>
-      <c r="T46" s="7"/>
-      <c r="U46" s="7"/>
-      <c r="V46" s="7"/>
-      <c r="W46" s="7"/>
-      <c r="X46" s="7"/>
-      <c r="Y46" s="7"/>
-      <c r="Z46" s="7"/>
-      <c r="AA46" s="7"/>
-    </row>
+    <row r="45" ht="15.75" customHeight="1">
+      <c r="A45" s="7"/>
+      <c r="B45" s="7"/>
+      <c r="C45" s="7"/>
+      <c r="D45" s="7"/>
+      <c r="E45" s="7"/>
+      <c r="F45" s="7"/>
+      <c r="G45" s="7"/>
+      <c r="H45" s="7"/>
+      <c r="I45" s="7"/>
+      <c r="J45" s="7"/>
+      <c r="K45" s="7"/>
+      <c r="L45" s="7"/>
+      <c r="M45" s="7"/>
+      <c r="N45" s="7"/>
+      <c r="O45" s="7"/>
+      <c r="P45" s="7"/>
+      <c r="Q45" s="7"/>
+      <c r="R45" s="7"/>
+      <c r="S45" s="7"/>
+      <c r="T45" s="7"/>
+      <c r="U45" s="7"/>
+      <c r="V45" s="7"/>
+      <c r="W45" s="7"/>
+      <c r="X45" s="7"/>
+      <c r="Y45" s="7"/>
+      <c r="Z45" s="7"/>
+      <c r="AA45" s="7"/>
+    </row>
+    <row r="46" ht="15.75" customHeight="1"/>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="7"/>
       <c r="B47" s="7"/>
       <c r="C47" s="3"/>
-      <c r="D47" s="16"/>
-      <c r="E47" s="16"/>
+      <c r="D47" s="17"/>
+      <c r="E47" s="17"/>
       <c r="F47" s="7"/>
-      <c r="G47" s="16"/>
+      <c r="G47" s="17"/>
       <c r="H47" s="7"/>
       <c r="I47" s="7"/>
-      <c r="J47" s="18"/>
+      <c r="J47" s="19"/>
       <c r="K47" s="7"/>
       <c r="L47" s="7"/>
       <c r="M47" s="7"/>
@@ -2534,13 +2640,13 @@
       <c r="A48" s="7"/>
       <c r="B48" s="7"/>
       <c r="C48" s="3"/>
-      <c r="D48" s="16"/>
-      <c r="E48" s="16"/>
+      <c r="D48" s="17"/>
+      <c r="E48" s="17"/>
       <c r="F48" s="7"/>
-      <c r="G48" s="16"/>
+      <c r="G48" s="17"/>
       <c r="H48" s="7"/>
       <c r="I48" s="7"/>
-      <c r="J48" s="7"/>
+      <c r="J48" s="19"/>
       <c r="K48" s="7"/>
       <c r="L48" s="7"/>
       <c r="M48" s="7"/>
@@ -2563,10 +2669,10 @@
       <c r="A49" s="7"/>
       <c r="B49" s="7"/>
       <c r="C49" s="3"/>
-      <c r="D49" s="16"/>
-      <c r="E49" s="16"/>
+      <c r="D49" s="17"/>
+      <c r="E49" s="17"/>
       <c r="F49" s="7"/>
-      <c r="G49" s="16"/>
+      <c r="G49" s="17"/>
       <c r="H49" s="7"/>
       <c r="I49" s="7"/>
       <c r="J49" s="7"/>
@@ -2588,7 +2694,35 @@
       <c r="Z49" s="7"/>
       <c r="AA49" s="7"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1"/>
+    <row r="50" ht="15.75" customHeight="1">
+      <c r="A50" s="7"/>
+      <c r="B50" s="7"/>
+      <c r="C50" s="3"/>
+      <c r="D50" s="17"/>
+      <c r="E50" s="17"/>
+      <c r="F50" s="7"/>
+      <c r="G50" s="17"/>
+      <c r="H50" s="7"/>
+      <c r="I50" s="7"/>
+      <c r="J50" s="7"/>
+      <c r="K50" s="7"/>
+      <c r="L50" s="7"/>
+      <c r="M50" s="7"/>
+      <c r="N50" s="7"/>
+      <c r="O50" s="7"/>
+      <c r="P50" s="7"/>
+      <c r="Q50" s="7"/>
+      <c r="R50" s="7"/>
+      <c r="S50" s="7"/>
+      <c r="T50" s="7"/>
+      <c r="U50" s="7"/>
+      <c r="V50" s="7"/>
+      <c r="W50" s="7"/>
+      <c r="X50" s="7"/>
+      <c r="Y50" s="7"/>
+      <c r="Z50" s="7"/>
+      <c r="AA50" s="7"/>
+    </row>
     <row r="51" ht="15.75" customHeight="1"/>
     <row r="52" ht="15.75" customHeight="1"/>
     <row r="53" ht="15.75" customHeight="1"/>
@@ -3541,7 +3675,11 @@
     <row r="1000" ht="15.75" customHeight="1"/>
     <row r="1001" ht="15.75" customHeight="1"/>
     <row r="1002" ht="15.75" customHeight="1"/>
+    <row r="1003" ht="15.75" customHeight="1"/>
   </sheetData>
+  <printOptions gridLines="1" horizontalCentered="1"/>
+  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageSetup fitToHeight="0" cellComments="atEnd" orientation="landscape" pageOrder="overThenDown"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>